<commit_message>
chore: update news radar report 2026-08-19
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-08-19.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-08-19.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,54 +446,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rising Impact Of Orphan Drugs And High-Cost Medications On Self-Funded Pharmacy Spend</t>
+          <t>UnitedHealthcare Expands Behavioral Coaching Access for 13 Million Commercial Members</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A growing concentration of pharmacy spend driven by orphan drugs and ultra-high-cost medications among a very small percentage of plan members has emerged as a major cost driver for self-funded employers. This trend severely threatens employer healthcare budgets by introducing unpredictable, catastrophic claims that standard stop-loss policies may not fully insulate. For pharmacy benefits managers, addressing this shift requires deploying advanced specialty drug containment strategies, robust utilization management, and targeted clinical oversight to protect plan sponsors from extreme financial volatility.</t>
+          <t>UnitedHealthcare has expanded its child and family behavioral coaching program to reach 13 million commercial members, addressing the growing demand for mental health support within employer-sponsored plans. This initiative matters because it highlights how major payers are proactively integrating specialized behavioral health benefits to improve overall employee wellness and curb downstream medical costs. For self-funded employers and benefit managers, this trend underscores the strategic value of offering comprehensive mental health solutions to attract talent and manage long-term healthcare utilization.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EIN News</t>
+          <t>Investing News Network</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tue, 18 Aug 2026 12:00:00 GMT</t>
+          <t>Wed, 19 Aug 2026 00:39:04 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxNcWxtMVF2bjBTVVA3aEoxS0kxamg1bTlET0ZoVGZEWU1fR2JlREFXaXR0U0hKd3hWVUFiay1qXzI5elV2ZHBMSm9BWTZPQzEwWWd5ZlNPU24ySDRhYnBiSGVnM3EwT1ZKMkhYSDZOMjBia2RZejU1dDRHZFdaeWcyNWdBZDF6Tk1MUHl3NVhCa3lUS1RCNmo5NVU4NUxhUzVhZkEwRXBQNFFIX2dheVAtWHlNWl9NZlZYbnNiVUh5SUZ5aC0wb1JCQ01SbGREQXhQUWZ2ZmlkZk8ybHUwWFd0WVhpS18wdw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Data-Driven Insights Outpace Cost Pressures in Employer Health Spending Decisions</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Recent industry data reveals that self-funded employers are shifting from reactive cost-cutting to data-driven decision-making when managing employee health and pharmacy benefits. This matters because relying on concrete analytics rather than general budget pressures allows organizations to target inefficiencies and specialty drug spend more effectively. For PBM partners and employee benefits leaders, this trend underscores the growing demand for transparent, data-backed solutions that prove return on investment and guide strategic plan design.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Insurance Business</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Tue, 18 Aug 2026 06:54:06 GMT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQX1VOdjh2ZGttSFh3QloxVExJODdZenBUeE00cG9XN0VGOVFHdXE0V1R3WFZhVkEtTDE5T0czb2dSU09lTDNNaEN1c0lDQUpzVno3N3dIdXVfVFVqcDVTaGFyZHYxNk1pWVQwS1RRWXBXUlpSSVNuSGM1YW1ROFdqbzRWQlVNZ0NkaGROTk1sZE1Td0hSZ1ZCVVJOU2E5MUVnVktVb05ZbnBMQmZ0WGhjVmNuWmN0OUdzZ3BZYWFKMUJMWEowclJSdk1XQ1NsMHotY0V2bg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxObEkzelFaWUZ6bXVfb0Mxb09MRnE4Vy1QVFJ5YjFCVjZxb1A5ZkxTaHMxQ0lZNGV5Yllwdmo4aEM1YTAzMjdQQmttV1ZfYVM1YnVzcHpoSVRPV1hQc09sMEluMmFPTmlOd2t3RzUxZndSdzg2bFRhaFBDQmc0Z2RBRjEwSWdHZEVXX2M2Z1VDZmtpQThKd0VRX09ROW1tYjdRcmd4Tjlpb3NReWNITXhKMEtyVVhjZjlPWDhzYmVqcFhuYkc3V1dPOFAtYw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>